<commit_message>
calibration updates week of 6/16
</commit_message>
<xml_diff>
--- a/InputData/elec/GBCGpUNR/Grid Bat Cap Growth per Unit Net Revenue.xlsx
+++ b/InputData/elec/GBCGpUNR/Grid Bat Cap Growth per Unit Net Revenue.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\elec\GBCGpUNR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\Mexico EPS\InputData\elec\GBCGpUNR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C74A81D-3725-4C8A-8875-8C49E5853CD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19432B33-6C8D-4964-ACE0-5A1544409700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="-1185" windowWidth="24240" windowHeight="13140" xr2:uid="{7E47E401-4FF2-4F75-986A-BA871D3584BD}"/>
+    <workbookView xWindow="30780" yWindow="2130" windowWidth="28245" windowHeight="12525" activeTab="1" xr2:uid="{7E47E401-4FF2-4F75-986A-BA871D3584BD}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="GBCGpUNR" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>GBPGpUNR Grid Battery Percent Growth per Unit Net Revenue</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t>MW per $/MWh net revenue</t>
+  </si>
+  <si>
+    <t>We multiplied the US value of 2000 by .08 to represent the ratio of the total power sector of MX to the US</t>
   </si>
 </sst>
 </file>
@@ -130,9 +133,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -170,7 +173,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -276,7 +279,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -418,7 +421,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -426,15 +429,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1BF9ED0-8E48-4355-BDAD-C352BC3B92D2}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -442,9 +445,14 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -458,12 +466,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="62.81640625" customWidth="1"/>
+    <col min="1" max="1" width="62.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -471,12 +479,13 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2">
-        <v>2000</v>
+        <f>2000*0.08</f>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -629,6 +638,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -637,20 +652,37 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB02944E-DC7D-4199-B8C9-3D27A285B2F4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB02944E-DC7D-4199-B8C9-3D27A285B2F4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2184511A-00A1-486A-B9C9-6904477248DA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07B0B04E-8B83-4177-93BE-766304BA5ACC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07B0B04E-8B83-4177-93BE-766304BA5ACC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2184511A-00A1-486A-B9C9-6904477248DA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>